<commit_message>
Trial 09: fix the raw data workbook Excel offered to recover; Excel icon on its download
Workbook: workbook.xml had firstSheet=1 with only one sheet (index 0), a
known trigger for Excel's repair prompt, and opened minimised; set
firstSheet=0, dropped minimized, removed 24 empty <v></v> on helper
formulas. All 3,770 cells and number formats unchanged; LibreOffice opens
and recalculates it. Also 06: Matt's 'genuine stakeholder (main ones)' and
ONLY in the inclusion rule.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Copilot_Excel_Raw_Data.xlsx
+++ b/Copilot_Excel_Raw_Data.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="1" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="8040" yWindow="3885" windowWidth="10245" windowHeight="7200" tabRatio="600" firstSheet="1" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="8040" yWindow="3885" windowWidth="10245" windowHeight="7200" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw data" sheetId="1" state="visible" r:id="rId1"/>
@@ -714,11 +714,9 @@
       </c>
       <c r="Y2" s="5">
         <f>SUMIF($B$2:$B$145,X2,$E$2:$E$145)</f>
-        <v/>
       </c>
       <c r="Z2" s="5">
         <f>SUMIF($B$2:$B$145,X2,$F$2:$F$145)</f>
-        <v/>
       </c>
     </row>
     <row r="3">
@@ -763,11 +761,9 @@
       </c>
       <c r="Y3" s="5">
         <f>SUMIF($B$2:$B$145,X3,$E$2:$E$145)</f>
-        <v/>
       </c>
       <c r="Z3" s="5">
         <f>SUMIF($B$2:$B$145,X3,$F$2:$F$145)</f>
-        <v/>
       </c>
     </row>
     <row r="4">
@@ -812,11 +808,9 @@
       </c>
       <c r="Y4" s="5">
         <f>SUMIF($B$2:$B$145,X4,$E$2:$E$145)</f>
-        <v/>
       </c>
       <c r="Z4" s="5">
         <f>SUMIF($B$2:$B$145,X4,$F$2:$F$145)</f>
-        <v/>
       </c>
     </row>
     <row r="5">
@@ -861,11 +855,9 @@
       </c>
       <c r="Y5" s="5">
         <f>SUMIF($B$2:$B$145,X5,$E$2:$E$145)</f>
-        <v/>
       </c>
       <c r="Z5" s="5">
         <f>SUMIF($B$2:$B$145,X5,$F$2:$F$145)</f>
-        <v/>
       </c>
     </row>
     <row r="6">
@@ -910,11 +902,9 @@
       </c>
       <c r="Y6" s="5">
         <f>SUMIF($B$2:$B$145,X6,$E$2:$E$145)</f>
-        <v/>
       </c>
       <c r="Z6" s="5">
         <f>SUMIF($B$2:$B$145,X6,$F$2:$F$145)</f>
-        <v/>
       </c>
     </row>
     <row r="7">
@@ -959,11 +949,9 @@
       </c>
       <c r="Y7" s="5">
         <f>SUMIF($B$2:$B$145,X7,$E$2:$E$145)</f>
-        <v/>
       </c>
       <c r="Z7" s="5">
         <f>SUMIF($B$2:$B$145,X7,$F$2:$F$145)</f>
-        <v/>
       </c>
     </row>
     <row r="8">
@@ -1008,11 +996,9 @@
       </c>
       <c r="Y8" s="5">
         <f>SUMIF($B$2:$B$145,X8,$E$2:$E$145)</f>
-        <v/>
       </c>
       <c r="Z8" s="5">
         <f>SUMIF($B$2:$B$145,X8,$F$2:$F$145)</f>
-        <v/>
       </c>
     </row>
     <row r="9">
@@ -1057,11 +1043,9 @@
       </c>
       <c r="Y9" s="5">
         <f>SUMIF($B$2:$B$145,X9,$E$2:$E$145)</f>
-        <v/>
       </c>
       <c r="Z9" s="5">
         <f>SUMIF($B$2:$B$145,X9,$F$2:$F$145)</f>
-        <v/>
       </c>
     </row>
     <row r="10">
@@ -1106,11 +1090,9 @@
       </c>
       <c r="Y10" s="5">
         <f>SUMIF($B$2:$B$145,X10,$E$2:$E$145)</f>
-        <v/>
       </c>
       <c r="Z10" s="5">
         <f>SUMIF($B$2:$B$145,X10,$F$2:$F$145)</f>
-        <v/>
       </c>
     </row>
     <row r="11">
@@ -1155,11 +1137,9 @@
       </c>
       <c r="Y11" s="5">
         <f>SUMIF($B$2:$B$145,X11,$E$2:$E$145)</f>
-        <v/>
       </c>
       <c r="Z11" s="5">
         <f>SUMIF($B$2:$B$145,X11,$F$2:$F$145)</f>
-        <v/>
       </c>
     </row>
     <row r="12">
@@ -1204,11 +1184,9 @@
       </c>
       <c r="Y12" s="5">
         <f>SUMIF($B$2:$B$145,X12,$E$2:$E$145)</f>
-        <v/>
       </c>
       <c r="Z12" s="5">
         <f>SUMIF($B$2:$B$145,X12,$F$2:$F$145)</f>
-        <v/>
       </c>
     </row>
     <row r="13">
@@ -1253,11 +1231,9 @@
       </c>
       <c r="Y13" s="5">
         <f>SUMIF($B$2:$B$145,X13,$E$2:$E$145)</f>
-        <v/>
       </c>
       <c r="Z13" s="5">
         <f>SUMIF($B$2:$B$145,X13,$F$2:$F$145)</f>
-        <v/>
       </c>
     </row>
     <row r="14">

</xml_diff>